<commit_message>
Se agrego lo de adrian
</commit_message>
<xml_diff>
--- a/salida.xlsx
+++ b/salida.xlsx
@@ -185,8 +185,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tabla_db" displayName="tabla_db" ref="A1:I2601" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I2601"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tabla_db" displayName="tabla_db" ref="A1:I2609" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I2609"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Dia"/>
@@ -203,8 +203,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tabla_pordia" displayName="tabla_pordia" ref="A1:H326" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:H326"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tabla_pordia" displayName="tabla_pordia" ref="A1:H327" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:H327"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Dia"/>
@@ -75982,6 +75982,238 @@
         <v>73</v>
       </c>
     </row>
+    <row r="2602">
+      <c r="A2602" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B2602" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2602" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2602" t="n">
+        <v>701</v>
+      </c>
+      <c r="E2602" t="n">
+        <v>778</v>
+      </c>
+      <c r="F2602" t="n">
+        <v>564</v>
+      </c>
+      <c r="G2602" t="n">
+        <v>214</v>
+      </c>
+      <c r="H2602" t="n">
+        <v>462</v>
+      </c>
+      <c r="I2602" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2603">
+      <c r="A2603" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B2603" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2603" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2603" t="n">
+        <v>248</v>
+      </c>
+      <c r="E2603" t="n">
+        <v>144</v>
+      </c>
+      <c r="F2603" t="n">
+        <v>143</v>
+      </c>
+      <c r="G2603" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2603" t="n">
+        <v>138</v>
+      </c>
+      <c r="I2603" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2604">
+      <c r="A2604" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B2604" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2604" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2604" t="n">
+        <v>953</v>
+      </c>
+      <c r="E2604" t="n">
+        <v>979</v>
+      </c>
+      <c r="F2604" t="n">
+        <v>817</v>
+      </c>
+      <c r="G2604" t="n">
+        <v>162</v>
+      </c>
+      <c r="H2604" t="n">
+        <v>797</v>
+      </c>
+      <c r="I2604" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2605">
+      <c r="A2605" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B2605" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2605" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2605" t="n">
+        <v>952</v>
+      </c>
+      <c r="E2605" t="n">
+        <v>894</v>
+      </c>
+      <c r="F2605" t="n">
+        <v>894</v>
+      </c>
+      <c r="G2605" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2605" t="n">
+        <v>869</v>
+      </c>
+      <c r="I2605" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2606">
+      <c r="A2606" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B2606" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2606" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2606" t="n">
+        <v>1031</v>
+      </c>
+      <c r="E2606" t="n">
+        <v>878</v>
+      </c>
+      <c r="F2606" t="n">
+        <v>646</v>
+      </c>
+      <c r="G2606" t="n">
+        <v>232</v>
+      </c>
+      <c r="H2606" t="n">
+        <v>544</v>
+      </c>
+      <c r="I2606" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2607">
+      <c r="A2607" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B2607" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2607" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2607" t="n">
+        <v>481</v>
+      </c>
+      <c r="E2607" t="n">
+        <v>908</v>
+      </c>
+      <c r="F2607" t="n">
+        <v>665</v>
+      </c>
+      <c r="G2607" t="n">
+        <v>243</v>
+      </c>
+      <c r="H2607" t="n">
+        <v>624</v>
+      </c>
+      <c r="I2607" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2608">
+      <c r="A2608" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B2608" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2608" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2608" t="n">
+        <v>285</v>
+      </c>
+      <c r="E2608" t="n">
+        <v>742</v>
+      </c>
+      <c r="F2608" t="n">
+        <v>348</v>
+      </c>
+      <c r="G2608" t="n">
+        <v>394</v>
+      </c>
+      <c r="H2608" t="n">
+        <v>308</v>
+      </c>
+      <c r="I2608" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2609">
+      <c r="A2609" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B2609" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2609" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2609" t="n">
+        <v>731</v>
+      </c>
+      <c r="E2609" t="n">
+        <v>805</v>
+      </c>
+      <c r="F2609" t="n">
+        <v>504</v>
+      </c>
+      <c r="G2609" t="n">
+        <v>301</v>
+      </c>
+      <c r="H2609" t="n">
+        <v>465</v>
+      </c>
+      <c r="I2609" t="n">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -84480,6 +84712,32 @@
       </c>
       <c r="H326" t="n">
         <v>326</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B327" t="s">
+        <v>20</v>
+      </c>
+      <c r="C327" t="n">
+        <v>5382</v>
+      </c>
+      <c r="D327" t="n">
+        <v>6128</v>
+      </c>
+      <c r="E327" t="n">
+        <v>4581</v>
+      </c>
+      <c r="F327" t="n">
+        <v>1547</v>
+      </c>
+      <c r="G327" t="n">
+        <v>4207</v>
+      </c>
+      <c r="H327" t="n">
+        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -87999,46 +88257,46 @@
         <v>46041</v>
       </c>
       <c r="B48" s="1" t="n">
-        <v>46043</v>
+        <v>46044</v>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>15731</v>
+        <v>21113</v>
       </c>
       <c r="E48" t="n">
-        <v>17777</v>
+        <v>23905</v>
       </c>
       <c r="F48" t="n">
-        <v>12020</v>
+        <v>16601</v>
       </c>
       <c r="G48" t="n">
-        <v>5757</v>
+        <v>7304</v>
       </c>
       <c r="H48" t="n">
-        <v>11173</v>
+        <v>15380</v>
       </c>
       <c r="I48" t="n">
-        <v>847</v>
+        <v>1221</v>
       </c>
       <c r="J48" t="n">
-        <v>5243.66666666667</v>
+        <v>5278.25</v>
       </c>
       <c r="K48" t="n">
-        <v>5925.66666666667</v>
+        <v>5976.25</v>
       </c>
       <c r="L48" t="n">
-        <v>4006.66666666667</v>
+        <v>4150.25</v>
       </c>
       <c r="M48" t="n">
-        <v>1919</v>
+        <v>1826</v>
       </c>
       <c r="N48" t="n">
-        <v>3724.33333333333</v>
+        <v>3845</v>
       </c>
       <c r="O48" t="n">
-        <v>282.333333333333</v>
+        <v>305.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>